<commit_message>
Santrfor mevkisi ST → SNT olarak Türkçeleştirildi (site + Excel)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veriler/Oyuncular ve İstatistikleri/Oyuncular ve İstatistikleri.xlsx
+++ b/Veriler/Oyuncular ve İstatistikleri/Oyuncular ve İstatistikleri.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>ST/MOO/SLK/SĞK</t>
+          <t>SNT/MOO/SLK/SĞK</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>ST/MOO/SLK/SĞK</t>
+          <t>SNT/MOO/SLK/SĞK</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>ST/MOO/SLK/SĞK</t>
+          <t>SNT/MOO/SLK/SĞK</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>MO/ST</t>
+          <t>MO/SNT</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Mevki sıralaması: SNT, SĞK, SLK, MOO, MO, MDO, STP, KL
- Tüm oyuncuların mevkileri yeni sıraya göre düzenlendi
- defaultPlayers, bilgi düzenleme formu, Firebase editleri
- Excel dosyası da güncellendi
- sortPositions() global fonksiyonu ile her yerde tutarlı sıralama

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veriler/Oyuncular ve İstatistikleri/Oyuncular ve İstatistikleri.xlsx
+++ b/Veriler/Oyuncular ve İstatistikleri/Oyuncular ve İstatistikleri.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>SNT/MOO/SLK/SĞK</t>
+          <t>SNT/SĞK/SLK/MOO</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>SNT/MOO/SLK/SĞK</t>
+          <t>SNT/SĞK/SLK/MOO</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>SNT/MOO/SLK/SĞK</t>
+          <t>SNT/SĞK/SLK/MOO</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>MO/SNT</t>
+          <t>SNT/MO</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>STP/MO/MDO</t>
+          <t>MO/MDO/STP</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>STP/MO/MDO</t>
+          <t>MO/MDO/STP</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">

</xml_diff>